<commit_message>
added supbase database and session form repeated column reduction
</commit_message>
<xml_diff>
--- a/demo-session-3-it-digital.xlsx
+++ b/demo-session-3-it-digital.xlsx
@@ -397,557 +397,213 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:D14"/>
   <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="5.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="28.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>TrnName</v>
+        <v>SN</v>
       </c>
       <c r="B1" t="str">
-        <v>Date</v>
+        <v>EnrollNo</v>
       </c>
       <c r="C1" t="str">
-        <v>Venue</v>
+        <v>EmployeeName</v>
       </c>
       <c r="D1" t="str">
-        <v>TimeFrom</v>
-      </c>
-      <c r="E1" t="str">
-        <v>TimeTo</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Trainer</v>
-      </c>
-      <c r="G1" t="str">
-        <v>TrainerDesignation</v>
-      </c>
-      <c r="H1" t="str">
-        <v>TrainerOrg</v>
-      </c>
-      <c r="I1" t="str">
-        <v>SN</v>
-      </c>
-      <c r="J1" t="str">
-        <v>EnrollNo</v>
-      </c>
-      <c r="K1" t="str">
-        <v>EmployeeName</v>
-      </c>
-      <c r="L1" t="str">
         <v>Designation</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-03-22</v>
+        <v>415056</v>
       </c>
       <c r="C2" t="str">
-        <v>Online - Zoom</v>
+        <v>Saleh Newaz</v>
       </c>
       <c r="D2" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E2" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G2" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H2" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2" t="str">
-        <v>415056</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Saleh Newaz</v>
-      </c>
-      <c r="L2" t="str">
         <v>Senior Executive</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-03-22</v>
+        <v>540423</v>
       </c>
       <c r="C3" t="str">
-        <v>Online - Zoom</v>
+        <v>Prince Mahmud</v>
       </c>
       <c r="D3" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E3" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G3" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H3" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3" t="str">
-        <v>540423</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Prince Mahmud</v>
-      </c>
-      <c r="L3" t="str">
         <v>Junior Executive</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-03-22</v>
+        <v>543696</v>
       </c>
       <c r="C4" t="str">
-        <v>Online - Zoom</v>
+        <v>S A F Md Ahad</v>
       </c>
       <c r="D4" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E4" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G4" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H4" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I4">
-        <v>3</v>
-      </c>
-      <c r="J4" t="str">
-        <v>543696</v>
-      </c>
-      <c r="K4" t="str">
-        <v>S A F Md Ahad</v>
-      </c>
-      <c r="L4" t="str">
         <v>Junior Executive</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A5">
+        <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-03-22</v>
+        <v>551243</v>
       </c>
       <c r="C5" t="str">
-        <v>Online - Zoom</v>
+        <v>S M Zahid Hasan</v>
       </c>
       <c r="D5" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E5" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G5" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H5" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5" t="str">
-        <v>551243</v>
-      </c>
-      <c r="K5" t="str">
-        <v>S M Zahid Hasan</v>
-      </c>
-      <c r="L5" t="str">
         <v>Executive</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A6">
+        <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-03-22</v>
+        <v>538499</v>
       </c>
       <c r="C6" t="str">
-        <v>Online - Zoom</v>
+        <v>Mohammad Asaduzzaman Riad</v>
       </c>
       <c r="D6" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E6" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G6" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H6" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6" t="str">
-        <v>538499</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Mohammad Asaduzzaman Riad</v>
-      </c>
-      <c r="L6" t="str">
         <v>Executive</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A7">
+        <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-03-22</v>
+        <v>533443</v>
       </c>
       <c r="C7" t="str">
-        <v>Online - Zoom</v>
+        <v>Md. Abdulla Al Mamun Sazal</v>
       </c>
       <c r="D7" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E7" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G7" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H7" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I7">
-        <v>6</v>
-      </c>
-      <c r="J7" t="str">
-        <v>533443</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Md. Abdulla Al Mamun Sazal</v>
-      </c>
-      <c r="L7" t="str">
         <v>Executive</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A8">
+        <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-03-22</v>
+        <v>549198</v>
       </c>
       <c r="C8" t="str">
-        <v>Online - Zoom</v>
+        <v>Md. Rabbi Rahman</v>
       </c>
       <c r="D8" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E8" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G8" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H8" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I8">
-        <v>7</v>
-      </c>
-      <c r="J8" t="str">
-        <v>549198</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Md. Rabbi Rahman</v>
-      </c>
-      <c r="L8" t="str">
         <v>Executive</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A9">
+        <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-03-22</v>
+        <v>538840</v>
       </c>
       <c r="C9" t="str">
-        <v>Online - Zoom</v>
+        <v>Md. Shohel Rana</v>
       </c>
       <c r="D9" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E9" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G9" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H9" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I9">
-        <v>8</v>
-      </c>
-      <c r="J9" t="str">
-        <v>538840</v>
-      </c>
-      <c r="K9" t="str">
-        <v>Md. Shohel Rana</v>
-      </c>
-      <c r="L9" t="str">
         <v>Junior Executive</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A10">
+        <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-03-22</v>
+        <v>479219</v>
       </c>
       <c r="C10" t="str">
-        <v>Online - Zoom</v>
+        <v>Estiak Ahmed</v>
       </c>
       <c r="D10" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E10" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G10" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H10" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I10">
-        <v>9</v>
-      </c>
-      <c r="J10" t="str">
-        <v>479219</v>
-      </c>
-      <c r="K10" t="str">
-        <v>Estiak Ahmed</v>
-      </c>
-      <c r="L10" t="str">
         <v>Executive</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A11">
+        <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-03-22</v>
+        <v>539355</v>
       </c>
       <c r="C11" t="str">
-        <v>Online - Zoom</v>
+        <v>Md Saymum Joynal</v>
       </c>
       <c r="D11" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E11" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G11" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H11" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I11">
-        <v>10</v>
-      </c>
-      <c r="J11" t="str">
-        <v>539355</v>
-      </c>
-      <c r="K11" t="str">
-        <v>Md Saymum Joynal</v>
-      </c>
-      <c r="L11" t="str">
         <v>Executive</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A12">
+        <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-03-22</v>
+        <v>514242</v>
       </c>
       <c r="C12" t="str">
-        <v>Online - Zoom</v>
+        <v>Mohammad Rakib Ahmed</v>
       </c>
       <c r="D12" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E12" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G12" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H12" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I12">
-        <v>11</v>
-      </c>
-      <c r="J12" t="str">
-        <v>514242</v>
-      </c>
-      <c r="K12" t="str">
-        <v>Mohammad Rakib Ahmed</v>
-      </c>
-      <c r="L12" t="str">
         <v>Junior Executive</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A13">
+        <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-03-22</v>
+        <v>540689</v>
       </c>
       <c r="C13" t="str">
-        <v>Online - Zoom</v>
+        <v>Imran Kaisar</v>
       </c>
       <c r="D13" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E13" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G13" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H13" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I13">
-        <v>12</v>
-      </c>
-      <c r="J13" t="str">
-        <v>540689</v>
-      </c>
-      <c r="K13" t="str">
-        <v>Imran Kaisar</v>
-      </c>
-      <c r="L13" t="str">
         <v>Senior Executive</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="str">
-        <v>IT &amp; Digital Transformation</v>
+      <c r="A14">
+        <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-03-22</v>
+        <v>529517</v>
       </c>
       <c r="C14" t="str">
-        <v>Online - Zoom</v>
+        <v>Rasel Rana</v>
       </c>
       <c r="D14" t="str">
-        <v>10:00 AM</v>
-      </c>
-      <c r="E14" t="str">
-        <v>12:00 PM</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Dr. Arif Hossain</v>
-      </c>
-      <c r="G14" t="str">
-        <v>IT Consultant</v>
-      </c>
-      <c r="H14" t="str">
-        <v>TechBridge Solutions Ltd.</v>
-      </c>
-      <c r="I14">
-        <v>13</v>
-      </c>
-      <c r="J14" t="str">
-        <v>529517</v>
-      </c>
-      <c r="K14" t="str">
-        <v>Rasel Rana</v>
-      </c>
-      <c r="L14" t="str">
         <v>Executive</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>